<commit_message>
Fix unit test: Add missing payment_method_mapping to mock ApplicationConfig
- Added PaymentMethodMappingConfig import to test_main.py
- Added payment_method_mapping attribute to mock configurations in TestCreateComponents
- Fixes AttributeError in create_components test after adding payment method mapping feature
- All 796 tests now passing with 90.41% coverage
- Applied ruff formatting fixes
</commit_message>
<xml_diff>
--- a/output/MERCADOPAGO_20250201.xlsx
+++ b/output/MERCADOPAGO_20250201.xlsx
@@ -476,7 +476,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1576,7 +1576,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1726,7 +1726,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -1976,7 +1976,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2026,7 +2026,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2176,7 +2176,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2451,7 +2451,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2601,7 +2601,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2626,7 +2626,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2651,7 +2651,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2726,7 +2726,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2776,7 +2776,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2876,7 +2876,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2926,7 +2926,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3101,7 +3101,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3126,7 +3126,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3176,7 +3176,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3226,7 +3226,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3276,7 +3276,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3301,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3376,7 +3376,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3476,7 +3476,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3551,7 +3551,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3626,7 +3626,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3651,7 +3651,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3676,7 +3676,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3701,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3726,7 +3726,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3776,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3801,7 +3801,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3826,7 +3826,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3851,7 +3851,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3876,7 +3876,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3926,7 +3926,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -3976,7 +3976,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4026,7 +4026,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4101,7 +4101,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4176,7 +4176,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4301,7 +4301,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4376,7 +4376,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4476,7 +4476,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4526,7 +4526,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4551,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4601,7 +4601,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4626,7 +4626,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4676,7 +4676,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4701,7 +4701,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4726,7 +4726,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4801,7 +4801,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4826,7 +4826,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4901,7 +4901,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4926,7 +4926,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4951,7 +4951,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -4976,7 +4976,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5001,7 +5001,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5026,7 +5026,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5051,7 +5051,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5076,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5101,7 +5101,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5151,7 +5151,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5201,7 +5201,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5251,7 +5251,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5351,7 +5351,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5376,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5401,7 +5401,7 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5426,7 +5426,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5451,7 +5451,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5476,7 +5476,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5501,7 +5501,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5526,7 +5526,7 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5551,7 +5551,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5576,7 +5576,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5601,7 +5601,7 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5626,7 +5626,7 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5651,7 +5651,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5676,7 +5676,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5701,7 +5701,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5751,7 +5751,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5776,7 +5776,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5801,7 +5801,7 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5851,7 +5851,7 @@
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5876,7 +5876,7 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5901,7 +5901,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5926,7 +5926,7 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5951,7 +5951,7 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6001,7 +6001,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6026,7 +6026,7 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6051,7 +6051,7 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6076,7 +6076,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6101,7 +6101,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6126,7 +6126,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6151,7 +6151,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6176,7 +6176,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6201,7 +6201,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6226,7 +6226,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6251,7 +6251,7 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6276,7 +6276,7 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6301,7 +6301,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6326,7 +6326,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6351,7 +6351,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6376,7 +6376,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6401,7 +6401,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6426,7 +6426,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6451,7 +6451,7 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6476,7 +6476,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6501,7 +6501,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6526,7 +6526,7 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6576,7 +6576,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6601,7 +6601,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6626,7 +6626,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6651,7 +6651,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6676,7 +6676,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6701,7 +6701,7 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6726,7 +6726,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6751,7 +6751,7 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6776,7 +6776,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6801,7 +6801,7 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6826,7 +6826,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6851,7 +6851,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6901,7 +6901,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6926,7 +6926,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6951,7 +6951,7 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -6976,7 +6976,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7001,7 +7001,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7026,7 +7026,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7051,7 +7051,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7076,7 +7076,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7101,7 +7101,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7126,7 +7126,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7151,7 +7151,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7176,7 +7176,7 @@
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7201,7 +7201,7 @@
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7226,7 +7226,7 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7276,7 +7276,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7301,7 +7301,7 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7326,7 +7326,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7351,7 +7351,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7401,7 +7401,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7426,7 +7426,7 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7451,7 +7451,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7476,7 +7476,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7501,7 +7501,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7526,7 +7526,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7551,7 +7551,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7576,7 +7576,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7601,7 +7601,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7626,7 +7626,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7651,7 +7651,7 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7676,7 +7676,7 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7701,7 +7701,7 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7726,7 +7726,7 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7751,7 +7751,7 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7776,7 +7776,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7801,7 +7801,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7826,7 +7826,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7876,7 +7876,7 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7901,7 +7901,7 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7951,7 +7951,7 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -7976,7 +7976,7 @@
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8001,7 +8001,7 @@
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8026,7 +8026,7 @@
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8051,7 +8051,7 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8076,7 +8076,7 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8101,7 +8101,7 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8126,7 +8126,7 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8151,7 +8151,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8176,7 +8176,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8201,7 +8201,7 @@
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8226,7 +8226,7 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8251,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8276,7 +8276,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8301,7 +8301,7 @@
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8326,7 +8326,7 @@
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8351,7 +8351,7 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8376,7 +8376,7 @@
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8401,7 +8401,7 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8426,7 +8426,7 @@
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8451,7 +8451,7 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8476,7 +8476,7 @@
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8501,7 +8501,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8526,7 +8526,7 @@
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8551,7 +8551,7 @@
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8576,7 +8576,7 @@
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8601,7 @@
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8626,7 +8626,7 @@
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8651,7 +8651,7 @@
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8676,7 +8676,7 @@
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8701,7 +8701,7 @@
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8726,7 +8726,7 @@
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8751,7 +8751,7 @@
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8776,7 +8776,7 @@
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8801,7 +8801,7 @@
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8826,7 +8826,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8851,7 +8851,7 @@
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8876,7 +8876,7 @@
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8901,7 +8901,7 @@
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8926,7 +8926,7 @@
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8951,7 +8951,7 @@
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -8976,7 +8976,7 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9001,7 +9001,7 @@
       </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9026,7 +9026,7 @@
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9051,7 +9051,7 @@
       </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9076,7 +9076,7 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9101,7 +9101,7 @@
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9126,7 +9126,7 @@
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9151,7 +9151,7 @@
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9176,7 +9176,7 @@
       </c>
       <c r="E350" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9201,7 +9201,7 @@
       </c>
       <c r="E351" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9226,7 +9226,7 @@
       </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9251,7 +9251,7 @@
       </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9276,7 +9276,7 @@
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9301,7 +9301,7 @@
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9326,7 +9326,7 @@
       </c>
       <c r="E356" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9351,7 +9351,7 @@
       </c>
       <c r="E357" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="E358" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9401,7 +9401,7 @@
       </c>
       <c r="E359" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9426,7 +9426,7 @@
       </c>
       <c r="E360" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9451,7 +9451,7 @@
       </c>
       <c r="E361" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9476,7 +9476,7 @@
       </c>
       <c r="E362" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9501,7 +9501,7 @@
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9526,7 +9526,7 @@
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9576,7 +9576,7 @@
       </c>
       <c r="E366" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9601,7 +9601,7 @@
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9626,7 +9626,7 @@
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9651,7 +9651,7 @@
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9676,7 +9676,7 @@
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9701,7 +9701,7 @@
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9726,7 +9726,7 @@
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9751,7 +9751,7 @@
       </c>
       <c r="E373" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9776,7 +9776,7 @@
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9801,7 +9801,7 @@
       </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9826,7 +9826,7 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9851,7 +9851,7 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9876,7 +9876,7 @@
       </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9901,7 +9901,7 @@
       </c>
       <c r="E379" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9926,7 +9926,7 @@
       </c>
       <c r="E380" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9951,7 +9951,7 @@
       </c>
       <c r="E381" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -9976,7 +9976,7 @@
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -10001,7 +10001,7 @@
       </c>
       <c r="E383" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -10026,7 +10026,7 @@
       </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -10051,7 +10051,7 @@
       </c>
       <c r="E385" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -10076,7 +10076,7 @@
       </c>
       <c r="E386" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -10101,7 +10101,7 @@
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -10126,7 +10126,7 @@
       </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -10151,7 +10151,7 @@
       </c>
       <c r="E389" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -10176,7 +10176,7 @@
       </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -10201,7 +10201,7 @@
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -10226,7 +10226,7 @@
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -10251,7 +10251,7 @@
       </c>
       <c r="E393" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -10276,7 +10276,7 @@
       </c>
       <c r="E394" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>
@@ -10301,7 +10301,7 @@
       </c>
       <c r="E395" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>MercadoPago_ENV_TEST</t>
         </is>
       </c>
     </row>

</xml_diff>